<commit_message>
update app.py / add files
</commit_message>
<xml_diff>
--- a/source/relatorios/2025/1-jan.xlsx
+++ b/source/relatorios/2025/1-jan.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t xml:space="preserve">Projeto</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t xml:space="preserve">CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t xml:space="preserve">CPBMF</t>
@@ -395,9 +392,7 @@
         <v>210</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="E7" s="1"/>
       <c r="F7" s="2"/>
       <c r="G7" s="1" t="n">
         <v>1</v>
@@ -405,7 +400,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>5</v>
@@ -426,7 +421,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>5</v>
@@ -443,7 +438,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>5</v>
@@ -460,7 +455,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>5</v>
@@ -477,7 +472,7 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>5</v>
@@ -494,7 +489,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>5</v>
@@ -517,7 +512,7 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>5</v>
@@ -538,7 +533,7 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>5</v>
@@ -557,7 +552,7 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>5</v>
@@ -574,7 +569,7 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>5</v>
@@ -593,7 +588,7 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>5</v>
@@ -614,7 +609,7 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>5</v>
@@ -637,7 +632,7 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>5</v>
@@ -660,7 +655,7 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>5</v>
@@ -677,7 +672,7 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>5</v>
@@ -694,7 +689,7 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>5</v>
@@ -711,7 +706,7 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>5</v>
@@ -728,7 +723,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>5</v>
@@ -747,7 +742,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>5</v>
@@ -768,7 +763,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>5</v>
@@ -787,7 +782,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>5</v>
@@ -808,7 +803,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>5</v>
@@ -825,7 +820,7 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>5</v>
@@ -842,7 +837,7 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>5</v>
@@ -859,7 +854,7 @@
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>5</v>
@@ -876,7 +871,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>5</v>
@@ -895,7 +890,7 @@
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>5</v>
@@ -912,7 +907,7 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>8</v>
@@ -923,7 +918,7 @@
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>3</v>

</xml_diff>